<commit_message>
feat: implementar envio nativo de imagenes usando sendImage de WAHA con fallback seguro
</commit_message>
<xml_diff>
--- a/documentos/base1.xlsx
+++ b/documentos/base1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\JONATHAN\Proyectos\BotEnvio_wsp\documentos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{823CA93F-0BAC-4CDF-B25C-46AA848C39D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976441AC-7C60-412E-84D5-55E1133F7A7E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1860" yWindow="1860" windowWidth="15375" windowHeight="7785" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Numero</t>
   </si>
@@ -33,13 +33,22 @@
     <t>Nombre</t>
   </si>
   <si>
-    <t>bety roxana</t>
-  </si>
-  <si>
     <t>Jonathan Vera</t>
   </si>
   <si>
     <t>ColdSolution</t>
+  </si>
+  <si>
+    <t>Maribel camello</t>
+  </si>
+  <si>
+    <t>Maicol Error</t>
+  </si>
+  <si>
+    <t>Eddy Error</t>
+  </si>
+  <si>
+    <t>Jaime Error</t>
   </si>
 </sst>
 </file>
@@ -357,7 +366,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -377,12 +386,12 @@
         <v>995799743</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>945430381</v>
+        <v>992609046</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -390,10 +399,34 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>992609046</v>
+        <v>988555500</v>
       </c>
       <c r="B4" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>945555888</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>633325698</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>945430381</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>